<commit_message>
modify xlsx and scenarios
</commit_message>
<xml_diff>
--- a/coretp/plans/svinval/SVINVAL_TP.xlsx
+++ b/coretp/plans/svinval/SVINVAL_TP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njoaquin/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njoaquin/Documents/Clean Test Plans/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D3CA660-5BA7-5B4D-9236-50BB3AF27447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82AEF59-1298-D349-AAE6-B39C14F80744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="820" windowWidth="34560" windowHeight="20440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -186,17 +186,48 @@
 2. Execute SFENCE.INVAL.IR -&gt; expect ILLEGAL_INSTRUCTION</t>
   </si>
   <si>
+    <t>U-mode fault test:
+1. Allocate memory with VALID, READ, WRITE flags
+2. Execute SINVAL.VMA -&gt; expect ILLEGAL_INSTRUCTION</t>
+  </si>
+  <si>
+    <t>S-mode with TVM=1 fault test:
+1. Allocate memory with VALID, READ, WRITE flags
+2. Set mstatus.TVM=1 (bit 20)
+3. Execute SINVAL.VMA -&gt; expect ILLEGAL_INSTRUCTION</t>
+  </si>
+  <si>
+    <t>U-mode no-fault test for SFENCE ops:
+1. Set mstatus.TVM=1 (bit 20)
+2. Execute SFENCE.W.INVAL -&gt; expect ILLEGAL_INSTRUCTION
+3. Execute SFENCE.INVAL.IR -&gt; expect ILLEGAL_INSTRUCTION</t>
+  </si>
+  <si>
+    <t>Non-consecutive invalidation instructions:
+1. Load from memory (bring PTE into TLB)
+2. Store to memory -&gt; expect STORE_AMO_PAGE_FAULT (no W bit)
+3. Read leaf PTE and save for comparison
+4. Set W bit in PTE (OR with 0x4)
+5. Write modified PTE back
+6. Execute SFENCE.W.INVAL
+7. Execute random arithmetic operation
+8. Execute SINVAL.VMA
+9. Execute random arithmetic operation
+10. Execute SFENCE.INVAL.IR
+11. Store to memory (should succeed)
+12. Read leaf PTE and verify it changed</t>
+  </si>
+  <si>
     <t>1. Load from memory (bring PTE into TLB)
 2. Store to memory -&gt; expect STORE_AMO_PAGE_FAULT (no W bit)
 3. Read leaf PTE and save for comparison
 4. Set W bit in PTE (OR with 0x4)
 5. Write modified PTE back
-6. Store to memory -&gt; expect STORE_AMO_PAGE_FAULT (TLB has old PTE)
-7. Execute SFENCE.W.INVAL
-8. Execute SINVAL.VMA
-9. Execute SFENCE.INVAL.IR
-10. Store to memory (should succeed)
-11. Read leaf PTE and verify it changed</t>
+6. Execute SFENCE.W.INVAL
+7. Execute SINVAL.VMA
+8. Execute SFENCE.INVAL.IR
+9. Store to memory (should succeed)
+10. Read leaf PTE and verify it changed</t>
   </si>
   <si>
     <t>Multiple VAs (VA1, VA2, VA3):
@@ -205,66 +236,25 @@
 3. Read all leaf PTEs
 4. Set W bit in all PTEs
 5. Write all PTEs back
-6. Store to all -&gt; expect STORE_AMO_PAGE_FAULT (TLB has old PTEs)
-7. Execute SFENCE.W.INVAL
-8. Execute SINVAL.VMA for VA1
-9. Execute SINVAL.VMA for VA2
-10. Execute SINVAL.VMA for VA3
-11. Execute SFENCE.INVAL.IR
-12. Store to all (should succeed)
-13. Verify all PTEs changed</t>
-  </si>
-  <si>
-    <t>Non-consecutive invalidation instructions:
-1. Load from memory (bring PTE into TLB)
-2. Store to memory -&gt; expect STORE_AMO_PAGE_FAULT (no W bit)
-3. Read leaf PTE and save for comparison
-4. Set W bit in PTE (OR with 0x4)
-5. Write modified PTE back
-6. Store to memory -&gt; expect STORE_AMO_PAGE_FAULT (TLB has old PTE)
-7. Execute SFENCE.W.INVAL
-8. Execute random arithmetic operation
-9. Execute SINVAL.VMA
-10. Execute random arithmetic operation
-11. Execute SFENCE.INVAL.IR
-12. Store to memory (should succeed)
-13. Read leaf PTE and verify it changed</t>
-  </si>
-  <si>
-    <t>U-mode fault test:
-1. Allocate memory with VALID, READ, WRITE flags
-2. Execute SINVAL.VMA -&gt; expect ILLEGAL_INSTRUCTION</t>
-  </si>
-  <si>
-    <t>S-mode with TVM=1 fault test:
-1. Allocate memory with VALID, READ, WRITE flags
-2. Set mstatus.TVM=1 (bit 20)
-3. Execute SINVAL.VMA -&gt; expect ILLEGAL_INSTRUCTION</t>
-  </si>
-  <si>
-    <t>U-mode no-fault test for SFENCE ops:
-1. Set mstatus.TVM=1 (bit 20)
-2. Execute SFENCE.W.INVAL -&gt; expect ILLEGAL_INSTRUCTION
-3. Execute SFENCE.INVAL.IR -&gt; expect ILLEGAL_INSTRUCTION</t>
+6. Execute SFENCE.W.INVAL
+7. Execute SINVAL.VMA for VA1
+8. Execute SINVAL.VMA for VA2
+9. Execute SINVAL.VMA for VA3
+10. Execute SFENCE.INVAL.IR
+11. Store to all (should succeed)
+12. Verify all PTEs changed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -404,38 +394,35 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -728,13 +715,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="10"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="9"/>
     </row>
     <row r="2" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -766,7 +753,7 @@
       <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="10" t="s">
         <v>34</v>
       </c>
     </row>
@@ -783,11 +770,11 @@
       <c r="D4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="204" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="170" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -800,11 +787,11 @@
       <c r="D5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="238" x14ac:dyDescent="0.2">
+      <c r="E5" s="10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="221" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -817,11 +804,11 @@
       <c r="D6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="255" x14ac:dyDescent="0.2">
+      <c r="E6" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="221" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -834,8 +821,8 @@
       <c r="D7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>38</v>
+      <c r="E7" s="10" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="51" x14ac:dyDescent="0.2">
@@ -852,7 +839,7 @@
         <v>25</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="68" x14ac:dyDescent="0.2">
@@ -869,7 +856,7 @@
         <v>28</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="85" x14ac:dyDescent="0.2">
@@ -886,7 +873,7 @@
         <v>32</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -915,15 +902,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100815CC0311B58BB469E58C0B9C6D5A1E3" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a19fa265d978d88ed6a7b13c74bee12e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e8037ae1-f799-41f0-b119-cbea2f4ab5d4" xmlns:ns3="b3c44bb9-2631-4400-93cf-11acafc6ee3a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1ebcff41a4cd7c30a8fef993265f2974" ns2:_="" ns3:_="">
     <xsd:import namespace="e8037ae1-f799-41f0-b119-cbea2f4ab5d4"/>
@@ -1172,6 +1150,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1184,14 +1171,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24752675-B760-43F1-B45D-4E8639F58F02}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A37CA4E4-13E9-4C3A-886D-534DD1626EFD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1210,6 +1189,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24752675-B760-43F1-B45D-4E8639F58F02}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F3B00C00-0ACA-41F1-AF8B-41145D6DFC1C}">
   <ds:schemaRefs>

</xml_diff>